<commit_message>
+ ADD fichiers = FIX dernier détail avant oral
</commit_message>
<xml_diff>
--- a/files/tableau_synthese_slam.xlsx
+++ b/files/tableau_synthese_slam.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28623"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\julie\Documents\MEGA\Supérieur\Stage SIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D6DFF35-3FF8-42A4-B2DC-BD72596DA2C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04284A93-8DC3-4595-8D07-95565DE4BC16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,14 +16,14 @@
     <sheet name="Tableau de synthèse Épreuve E4" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Tableau de synthèse Épreuve E4'!$A$1:$H$35</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Tableau de synthèse Épreuve E4'!$A$1:$H$36</definedName>
   </definedNames>
   <calcPr calcId="101716"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="55">
   <si>
     <t>Gérer le patrimoine informatique</t>
   </si>
@@ -142,34 +142,88 @@
     <t>Faire des points sur le projet, liste des taches (github)</t>
   </si>
   <si>
-    <t>Site Filmotech</t>
-  </si>
-  <si>
-    <t>Site "Le Grand Berger"</t>
-  </si>
-  <si>
     <t>Veille technologique</t>
   </si>
   <si>
     <t>2023-2025</t>
   </si>
   <si>
-    <t>Profil LinkedIn/Instagram</t>
-  </si>
-  <si>
-    <t>2022-25</t>
-  </si>
-  <si>
-    <t>Création d'un dashboard interne à l'entreprise</t>
-  </si>
-  <si>
-    <t>Création portfolio (identité, siteweb)</t>
-  </si>
-  <si>
     <t>N° candidat : 02047356179</t>
   </si>
   <si>
     <t>Adresse URL du portfolio : htpps://juliengournay.fr</t>
+  </si>
+  <si>
+    <t>Parcours de certification</t>
+  </si>
+  <si>
+    <t>2024-2025</t>
+  </si>
+  <si>
+    <t>SIO - Mise en place et configuration du service GLPI (VM)</t>
+  </si>
+  <si>
+    <t>SIO 1 - Projet : Création d'une site web "Le Grand Berger"</t>
+  </si>
+  <si>
+    <t>SIO 1 - Réalisation : Création d'un site web "Filmotech"</t>
+  </si>
+  <si>
+    <t>SIO 2 - Projet : Création d'un site web et d'un client lourd "Marie Team"</t>
+  </si>
+  <si>
+    <t>Réalisation d'un portfolio (avec base de données)</t>
+  </si>
+  <si>
+    <t>Réalisation d'un dashboard interne à l'entreprise sous Symfony</t>
+  </si>
+  <si>
+    <t>SIO 1 - Création d'une machine virtuel sous Débian</t>
+  </si>
+  <si>
+    <t>Utilisation de Github</t>
+  </si>
+  <si>
+    <t>Réalisation d'une billetterie sous Django</t>
+  </si>
+  <si>
+    <t>Utilisation d'un système de ticket d'incidence, surveillance matériels (GLPI)</t>
+  </si>
+  <si>
+    <t>fev-25</t>
+  </si>
+  <si>
+    <t>Bien choissir ses mots de passe</t>
+  </si>
+  <si>
+    <t>Ma présence en ligne</t>
+  </si>
+  <si>
+    <t>Conception de maquette pour la billeterie et mail</t>
+  </si>
+  <si>
+    <t>Mise en place d'une base de connaissance</t>
+  </si>
+  <si>
+    <t>SIO 2 - Tutoriel d'installation et configuration de HAProxy</t>
+  </si>
+  <si>
+    <t>Centralisation et système de monitoring</t>
+  </si>
+  <si>
+    <t>Compte rendu sur l'utilsation du système de monitoring</t>
+  </si>
+  <si>
+    <t>Création d'un environnement de développement (WSL)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Utilisation de GitHub </t>
+  </si>
+  <si>
+    <t>Tutoriel sur la procédure d'utilisation de la billetterie</t>
+  </si>
+  <si>
+    <t>Norme Gestion sémantique de version</t>
   </si>
 </sst>
 </file>
@@ -179,7 +233,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$€-1]_-;\-* #,##0.00\ [$€-1]_-;_-* &quot;-&quot;??\ [$€-1]_-"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="15">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -254,6 +308,18 @@
       <family val="2"/>
       <charset val="2"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <color theme="9"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FF00B050"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -269,7 +335,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="26">
+  <borders count="27">
     <border>
       <left/>
       <right/>
@@ -374,51 +440,6 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="medium">
-        <color theme="2" tint="-0.749992370372631"/>
-      </left>
-      <right style="thin">
-        <color theme="2" tint="-0.749992370372631"/>
-      </right>
-      <top style="thin">
-        <color theme="2" tint="-0.749992370372631"/>
-      </top>
-      <bottom style="medium">
-        <color theme="2" tint="-0.749992370372631"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="2" tint="-0.749992370372631"/>
-      </left>
-      <right style="thin">
-        <color theme="2" tint="-0.749992370372631"/>
-      </right>
-      <top style="thin">
-        <color theme="2" tint="-0.749992370372631"/>
-      </top>
-      <bottom style="medium">
-        <color theme="2" tint="-0.749992370372631"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="2" tint="-0.749992370372631"/>
-      </left>
-      <right style="medium">
-        <color theme="2" tint="-0.749992370372631"/>
-      </right>
-      <top style="thin">
-        <color theme="2" tint="-0.749992370372631"/>
-      </top>
-      <bottom style="medium">
-        <color theme="2" tint="-0.749992370372631"/>
-      </bottom>
-      <diagonal/>
-    </border>
     <border diagonalDown="1">
       <left style="medium">
         <color theme="2" tint="-0.749992370372631"/>
@@ -613,6 +634,58 @@
       <top style="thin">
         <color theme="2" tint="-0.749992370372631"/>
       </top>
+      <bottom style="thin">
+        <color theme="2" tint="-0.749992370372631"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color theme="2" tint="-0.749992370372631"/>
+      </left>
+      <right style="thin">
+        <color theme="2" tint="-0.749992370372631"/>
+      </right>
+      <top style="thin">
+        <color theme="2" tint="-0.749992370372631"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color theme="2" tint="-0.749992370372631"/>
+      </left>
+      <right style="thin">
+        <color theme="2" tint="-0.749992370372631"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color theme="2" tint="-0.749992370372631"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="2" tint="-0.749992370372631"/>
+      </left>
+      <right style="thin">
+        <color theme="2" tint="-0.749992370372631"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color theme="2" tint="-0.749992370372631"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="2" tint="-0.749992370372631"/>
+      </left>
+      <right style="medium">
+        <color theme="2" tint="-0.749992370372631"/>
+      </right>
+      <top/>
       <bottom style="thin">
         <color theme="2" tint="-0.749992370372631"/>
       </bottom>
@@ -623,7 +696,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -646,23 +719,17 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -676,34 +743,43 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="17" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="17" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -718,20 +794,47 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -739,23 +842,23 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1065,94 +1168,94 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AQ81"/>
+  <dimension ref="A1:AQ82"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.88671875" defaultRowHeight="13.2"/>
   <cols>
     <col min="1" max="1" width="70.44140625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="10.88671875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="14.44140625" style="1" customWidth="1"/>
     <col min="3" max="8" width="18.6640625" style="1" customWidth="1"/>
     <col min="9" max="43" width="11.44140625" customWidth="1"/>
     <col min="44" max="16384" width="10.88671875" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:43" ht="39.9" customHeight="1">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="29" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
-      <c r="E1" s="28"/>
-      <c r="F1" s="28"/>
-      <c r="G1" s="28" t="s">
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
+      <c r="E1" s="29"/>
+      <c r="F1" s="29"/>
+      <c r="G1" s="29" t="s">
         <v>22</v>
       </c>
-      <c r="H1" s="28"/>
+      <c r="H1" s="29"/>
     </row>
     <row r="2" spans="1:43" ht="41.1" customHeight="1" thickBot="1">
-      <c r="A2" s="28" t="s">
+      <c r="A2" s="29" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="28"/>
-      <c r="C2" s="28"/>
-      <c r="D2" s="28"/>
-      <c r="E2" s="28"/>
-      <c r="F2" s="28"/>
-      <c r="G2" s="28"/>
-      <c r="H2" s="28"/>
+      <c r="B2" s="29"/>
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="29"/>
+      <c r="F2" s="29"/>
+      <c r="G2" s="29"/>
+      <c r="H2" s="29"/>
     </row>
     <row r="3" spans="1:43" ht="39.9" customHeight="1">
-      <c r="A3" s="37" t="s">
+      <c r="A3" s="44" t="s">
         <v>23</v>
       </c>
-      <c r="B3" s="38"/>
-      <c r="C3" s="38"/>
-      <c r="D3" s="38"/>
-      <c r="E3" s="39"/>
-      <c r="F3" s="43" t="s">
-        <v>35</v>
-      </c>
-      <c r="G3" s="38"/>
-      <c r="H3" s="44"/>
+      <c r="B3" s="45"/>
+      <c r="C3" s="45"/>
+      <c r="D3" s="45"/>
+      <c r="E3" s="46"/>
+      <c r="F3" s="47" t="s">
+        <v>29</v>
+      </c>
+      <c r="G3" s="45"/>
+      <c r="H3" s="48"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
     </row>
     <row r="4" spans="1:43" ht="39.9" customHeight="1">
-      <c r="A4" s="40" t="s">
+      <c r="A4" s="41" t="s">
         <v>24</v>
       </c>
-      <c r="B4" s="41"/>
-      <c r="C4" s="41"/>
-      <c r="D4" s="41"/>
-      <c r="E4" s="42"/>
-      <c r="F4" s="14" t="s">
+      <c r="B4" s="42"/>
+      <c r="C4" s="42"/>
+      <c r="D4" s="42"/>
+      <c r="E4" s="43"/>
+      <c r="F4" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="G4" s="15" t="s">
+      <c r="G4" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="H4" s="21" t="s">
+      <c r="H4" s="17" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="5" spans="1:43" ht="39.9" customHeight="1" thickBot="1">
-      <c r="A5" s="40" t="s">
-        <v>36</v>
-      </c>
-      <c r="B5" s="41"/>
-      <c r="C5" s="41"/>
-      <c r="D5" s="41"/>
-      <c r="E5" s="42"/>
-      <c r="F5" s="40"/>
-      <c r="G5" s="41"/>
-      <c r="H5" s="41"/>
+      <c r="A5" s="41" t="s">
+        <v>30</v>
+      </c>
+      <c r="B5" s="42"/>
+      <c r="C5" s="42"/>
+      <c r="D5" s="42"/>
+      <c r="E5" s="43"/>
+      <c r="F5" s="41"/>
+      <c r="G5" s="42"/>
+      <c r="H5" s="42"/>
     </row>
     <row r="6" spans="1:43" ht="90" customHeight="1">
-      <c r="A6" s="26" t="s">
+      <c r="A6" s="27" t="s">
         <v>17</v>
       </c>
-      <c r="B6" s="35" t="s">
+      <c r="B6" s="39" t="s">
         <v>18</v>
       </c>
       <c r="C6" s="6" t="s">
@@ -1175,8 +1278,8 @@
       </c>
     </row>
     <row r="7" spans="1:43" s="2" customFormat="1" ht="324.89999999999998" customHeight="1" thickBot="1">
-      <c r="A7" s="27"/>
-      <c r="B7" s="36"/>
+      <c r="A7" s="28"/>
+      <c r="B7" s="40"/>
       <c r="C7" s="8" t="s">
         <v>9</v>
       </c>
@@ -1232,16 +1335,16 @@
       <c r="AQ7"/>
     </row>
     <row r="8" spans="1:43" s="2" customFormat="1" ht="17.399999999999999">
-      <c r="A8" s="29" t="s">
+      <c r="A8" s="30" t="s">
         <v>16</v>
       </c>
-      <c r="B8" s="30"/>
-      <c r="C8" s="30"/>
-      <c r="D8" s="30"/>
-      <c r="E8" s="30"/>
-      <c r="F8" s="30"/>
-      <c r="G8" s="30"/>
-      <c r="H8" s="31"/>
+      <c r="B8" s="31"/>
+      <c r="C8" s="31"/>
+      <c r="D8" s="31"/>
+      <c r="E8" s="31"/>
+      <c r="F8" s="31"/>
+      <c r="G8" s="31"/>
+      <c r="H8" s="32"/>
       <c r="I8"/>
       <c r="J8"/>
       <c r="K8"/>
@@ -1280,17 +1383,17 @@
     </row>
     <row r="9" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1">
       <c r="A9" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="B9" s="22">
+        <v>35</v>
+      </c>
+      <c r="B9" s="20">
         <v>45383</v>
       </c>
-      <c r="C9" s="16"/>
-      <c r="D9" s="17"/>
-      <c r="E9" s="17"/>
-      <c r="F9" s="23"/>
-      <c r="G9" s="17"/>
-      <c r="H9" s="18"/>
+      <c r="C9" s="14"/>
+      <c r="D9" s="15"/>
+      <c r="E9" s="15"/>
+      <c r="F9" s="18"/>
+      <c r="G9" s="15"/>
+      <c r="H9" s="16"/>
       <c r="I9"/>
       <c r="J9"/>
       <c r="K9"/>
@@ -1329,17 +1432,17 @@
     </row>
     <row r="10" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1">
       <c r="A10" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="B10" s="10">
+        <v>34</v>
+      </c>
+      <c r="B10" s="21">
         <v>2024</v>
       </c>
-      <c r="C10" s="17"/>
-      <c r="D10" s="17"/>
-      <c r="E10" s="17"/>
-      <c r="F10" s="23"/>
-      <c r="G10" s="17"/>
-      <c r="H10" s="18"/>
+      <c r="C10" s="15"/>
+      <c r="D10" s="15"/>
+      <c r="E10" s="18"/>
+      <c r="F10" s="18"/>
+      <c r="G10" s="15"/>
+      <c r="H10" s="16"/>
       <c r="I10"/>
       <c r="J10"/>
       <c r="K10"/>
@@ -1378,17 +1481,17 @@
     </row>
     <row r="11" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1">
       <c r="A11" s="11" t="s">
-        <v>34</v>
-      </c>
-      <c r="B11" s="10">
-        <v>2023</v>
-      </c>
-      <c r="C11" s="17"/>
-      <c r="D11" s="23"/>
-      <c r="E11" s="17"/>
-      <c r="F11" s="17"/>
-      <c r="G11" s="17"/>
-      <c r="H11" s="24"/>
+        <v>37</v>
+      </c>
+      <c r="B11" s="21" t="s">
+        <v>28</v>
+      </c>
+      <c r="C11" s="18"/>
+      <c r="D11" s="49"/>
+      <c r="E11" s="18"/>
+      <c r="F11" s="15"/>
+      <c r="G11" s="18"/>
+      <c r="H11" s="19"/>
       <c r="I11"/>
       <c r="J11"/>
       <c r="K11"/>
@@ -1427,17 +1530,17 @@
     </row>
     <row r="12" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1">
       <c r="A12" s="11" t="s">
-        <v>31</v>
-      </c>
-      <c r="B12" s="25" t="s">
-        <v>32</v>
-      </c>
-      <c r="C12" s="17"/>
-      <c r="D12" s="17"/>
-      <c r="E12" s="17"/>
-      <c r="F12" s="17"/>
-      <c r="G12" s="17"/>
-      <c r="H12" s="24"/>
+        <v>47</v>
+      </c>
+      <c r="B12" s="21">
+        <v>2025</v>
+      </c>
+      <c r="C12" s="18"/>
+      <c r="D12" s="15"/>
+      <c r="E12" s="15"/>
+      <c r="F12" s="15"/>
+      <c r="G12" s="18"/>
+      <c r="H12" s="53"/>
       <c r="I12"/>
       <c r="J12"/>
       <c r="K12"/>
@@ -1475,14 +1578,18 @@
       <c r="AQ12"/>
     </row>
     <row r="13" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1">
-      <c r="A13" s="11"/>
-      <c r="B13" s="10"/>
-      <c r="C13" s="17"/>
-      <c r="D13" s="17"/>
-      <c r="E13" s="17"/>
-      <c r="F13" s="17"/>
-      <c r="G13" s="17"/>
-      <c r="H13" s="18"/>
+      <c r="A13" s="50" t="s">
+        <v>36</v>
+      </c>
+      <c r="B13" s="21" t="s">
+        <v>32</v>
+      </c>
+      <c r="C13" s="51"/>
+      <c r="D13" s="15"/>
+      <c r="E13" s="52"/>
+      <c r="F13" s="18"/>
+      <c r="G13" s="18"/>
+      <c r="H13" s="16"/>
       <c r="I13"/>
       <c r="J13"/>
       <c r="K13"/>
@@ -1520,14 +1627,18 @@
       <c r="AQ13"/>
     </row>
     <row r="14" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1">
-      <c r="A14" s="11"/>
-      <c r="B14" s="10"/>
-      <c r="C14" s="17"/>
-      <c r="D14" s="17"/>
-      <c r="E14" s="17"/>
-      <c r="F14" s="17"/>
-      <c r="G14" s="17"/>
-      <c r="H14" s="18"/>
+      <c r="A14" s="50" t="s">
+        <v>33</v>
+      </c>
+      <c r="B14" s="21" t="s">
+        <v>32</v>
+      </c>
+      <c r="C14" s="18"/>
+      <c r="D14" s="54"/>
+      <c r="E14" s="15"/>
+      <c r="F14" s="15"/>
+      <c r="G14" s="15"/>
+      <c r="H14" s="16"/>
       <c r="I14"/>
       <c r="J14"/>
       <c r="K14"/>
@@ -1565,14 +1676,18 @@
       <c r="AQ14"/>
     </row>
     <row r="15" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1">
-      <c r="A15" s="11"/>
-      <c r="B15" s="10"/>
-      <c r="C15" s="17"/>
-      <c r="D15" s="17"/>
-      <c r="E15" s="17"/>
-      <c r="F15" s="17"/>
-      <c r="G15" s="17"/>
-      <c r="H15" s="18"/>
+      <c r="A15" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="B15" s="21">
+        <v>2023</v>
+      </c>
+      <c r="C15" s="18"/>
+      <c r="D15" s="15"/>
+      <c r="E15" s="15"/>
+      <c r="F15" s="15"/>
+      <c r="G15" s="18"/>
+      <c r="H15" s="16"/>
       <c r="I15"/>
       <c r="J15"/>
       <c r="K15"/>
@@ -1610,14 +1725,18 @@
       <c r="AQ15"/>
     </row>
     <row r="16" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1">
-      <c r="A16" s="11"/>
-      <c r="B16" s="10"/>
-      <c r="C16" s="17"/>
-      <c r="D16" s="17"/>
-      <c r="E16" s="17"/>
-      <c r="F16" s="17"/>
-      <c r="G16" s="17"/>
-      <c r="H16" s="18"/>
+      <c r="A16" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="B16" s="21">
+        <v>2025</v>
+      </c>
+      <c r="C16" s="18"/>
+      <c r="D16" s="15"/>
+      <c r="E16" s="15"/>
+      <c r="F16" s="15"/>
+      <c r="G16" s="18"/>
+      <c r="H16" s="16"/>
       <c r="I16"/>
       <c r="J16"/>
       <c r="K16"/>
@@ -1655,14 +1774,18 @@
       <c r="AQ16"/>
     </row>
     <row r="17" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1">
-      <c r="A17" s="11"/>
-      <c r="B17" s="10"/>
-      <c r="C17" s="17"/>
-      <c r="D17" s="17"/>
-      <c r="E17" s="17"/>
-      <c r="F17" s="17"/>
-      <c r="G17" s="17"/>
-      <c r="H17" s="18"/>
+      <c r="A17" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="B17" s="21">
+        <v>2025</v>
+      </c>
+      <c r="C17" s="18"/>
+      <c r="D17" s="15"/>
+      <c r="E17" s="15"/>
+      <c r="F17" s="15"/>
+      <c r="G17" s="52"/>
+      <c r="H17" s="16"/>
       <c r="I17"/>
       <c r="J17"/>
       <c r="K17"/>
@@ -1701,17 +1824,17 @@
     </row>
     <row r="18" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1">
       <c r="A18" s="11" t="s">
-        <v>29</v>
-      </c>
-      <c r="B18" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="C18" s="17"/>
-      <c r="D18" s="17"/>
-      <c r="E18" s="17"/>
-      <c r="F18" s="17"/>
-      <c r="G18" s="17"/>
-      <c r="H18" s="18"/>
+        <v>40</v>
+      </c>
+      <c r="B18" s="21">
+        <v>2024</v>
+      </c>
+      <c r="C18" s="18"/>
+      <c r="D18" s="18"/>
+      <c r="E18" s="15"/>
+      <c r="F18" s="15"/>
+      <c r="G18" s="15"/>
+      <c r="H18" s="16"/>
       <c r="I18"/>
       <c r="J18"/>
       <c r="K18"/>
@@ -1748,17 +1871,19 @@
       <c r="AP18"/>
       <c r="AQ18"/>
     </row>
-    <row r="19" spans="1:43" s="2" customFormat="1" ht="17.399999999999999">
-      <c r="A19" s="32" t="s">
-        <v>19</v>
-      </c>
-      <c r="B19" s="33"/>
-      <c r="C19" s="33"/>
-      <c r="D19" s="33"/>
-      <c r="E19" s="33"/>
-      <c r="F19" s="33"/>
-      <c r="G19" s="33"/>
-      <c r="H19" s="34"/>
+    <row r="19" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1">
+      <c r="A19" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="B19" s="21" t="s">
+        <v>28</v>
+      </c>
+      <c r="C19" s="15"/>
+      <c r="D19" s="15"/>
+      <c r="E19" s="15"/>
+      <c r="F19" s="15"/>
+      <c r="G19" s="15"/>
+      <c r="H19" s="19"/>
       <c r="I19"/>
       <c r="J19"/>
       <c r="K19"/>
@@ -1797,17 +1922,17 @@
     </row>
     <row r="20" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1">
       <c r="A20" s="11" t="s">
-        <v>25</v>
-      </c>
-      <c r="B20" s="22">
-        <v>45413</v>
-      </c>
-      <c r="C20" s="17"/>
-      <c r="D20" s="17"/>
-      <c r="E20" s="17"/>
-      <c r="F20" s="17"/>
-      <c r="G20" s="23"/>
-      <c r="H20" s="18"/>
+        <v>44</v>
+      </c>
+      <c r="B20" s="20">
+        <v>45748</v>
+      </c>
+      <c r="C20" s="18"/>
+      <c r="D20" s="15"/>
+      <c r="E20" s="15"/>
+      <c r="F20" s="15"/>
+      <c r="G20" s="18"/>
+      <c r="H20" s="16"/>
       <c r="I20"/>
       <c r="J20"/>
       <c r="K20"/>
@@ -1845,18 +1970,18 @@
       <c r="AQ20"/>
     </row>
     <row r="21" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1">
-      <c r="A21" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="B21" s="22">
-        <v>45413</v>
-      </c>
-      <c r="C21" s="17"/>
-      <c r="D21" s="17"/>
-      <c r="E21" s="17"/>
-      <c r="F21" s="23"/>
-      <c r="G21" s="17"/>
-      <c r="H21" s="18"/>
+      <c r="A21" s="50" t="s">
+        <v>45</v>
+      </c>
+      <c r="B21" s="20" t="s">
+        <v>28</v>
+      </c>
+      <c r="C21" s="15"/>
+      <c r="D21" s="15"/>
+      <c r="E21" s="52"/>
+      <c r="F21" s="15"/>
+      <c r="G21" s="15"/>
+      <c r="H21" s="19"/>
       <c r="I21"/>
       <c r="J21"/>
       <c r="K21"/>
@@ -1894,18 +2019,18 @@
       <c r="AQ21"/>
     </row>
     <row r="22" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1">
-      <c r="A22" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="B22" s="22">
-        <v>45413</v>
-      </c>
-      <c r="C22" s="17"/>
-      <c r="D22" s="17"/>
-      <c r="E22" s="17"/>
-      <c r="F22" s="17"/>
-      <c r="G22" s="17"/>
-      <c r="H22" s="18"/>
+      <c r="A22" s="50" t="s">
+        <v>27</v>
+      </c>
+      <c r="B22" s="21" t="s">
+        <v>28</v>
+      </c>
+      <c r="C22" s="15"/>
+      <c r="D22" s="15"/>
+      <c r="E22" s="15"/>
+      <c r="F22" s="15"/>
+      <c r="G22" s="15"/>
+      <c r="H22" s="19"/>
       <c r="I22"/>
       <c r="J22"/>
       <c r="K22"/>
@@ -1942,15 +2067,17 @@
       <c r="AP22"/>
       <c r="AQ22"/>
     </row>
-    <row r="23" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1">
-      <c r="A23" s="11"/>
-      <c r="B23" s="10"/>
-      <c r="C23" s="17"/>
-      <c r="D23" s="17"/>
-      <c r="E23" s="17"/>
-      <c r="F23" s="17"/>
-      <c r="G23" s="17"/>
-      <c r="H23" s="18"/>
+    <row r="23" spans="1:43" s="2" customFormat="1" ht="17.399999999999999">
+      <c r="A23" s="33" t="s">
+        <v>19</v>
+      </c>
+      <c r="B23" s="34"/>
+      <c r="C23" s="34"/>
+      <c r="D23" s="34"/>
+      <c r="E23" s="34"/>
+      <c r="F23" s="34"/>
+      <c r="G23" s="34"/>
+      <c r="H23" s="35"/>
       <c r="I23"/>
       <c r="J23"/>
       <c r="K23"/>
@@ -1988,14 +2115,18 @@
       <c r="AQ23"/>
     </row>
     <row r="24" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1">
-      <c r="A24" s="11"/>
-      <c r="B24" s="10"/>
-      <c r="C24" s="17"/>
-      <c r="D24" s="17"/>
-      <c r="E24" s="17"/>
-      <c r="F24" s="17"/>
-      <c r="G24" s="17"/>
-      <c r="H24" s="18"/>
+      <c r="A24" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="B24" s="20">
+        <v>45413</v>
+      </c>
+      <c r="C24" s="15"/>
+      <c r="D24" s="18"/>
+      <c r="E24" s="15"/>
+      <c r="F24" s="15"/>
+      <c r="G24" s="18"/>
+      <c r="H24" s="16"/>
       <c r="I24"/>
       <c r="J24"/>
       <c r="K24"/>
@@ -2033,14 +2164,18 @@
       <c r="AQ24"/>
     </row>
     <row r="25" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1">
-      <c r="A25" s="11"/>
-      <c r="B25" s="10"/>
-      <c r="C25" s="17"/>
-      <c r="D25" s="17"/>
-      <c r="E25" s="17"/>
-      <c r="F25" s="17"/>
-      <c r="G25" s="17"/>
-      <c r="H25" s="18"/>
+      <c r="A25" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="B25" s="20">
+        <v>45413</v>
+      </c>
+      <c r="C25" s="18"/>
+      <c r="D25" s="15"/>
+      <c r="E25" s="15"/>
+      <c r="F25" s="18"/>
+      <c r="G25" s="15"/>
+      <c r="H25" s="16"/>
       <c r="I25"/>
       <c r="J25"/>
       <c r="K25"/>
@@ -2078,14 +2213,18 @@
       <c r="AQ25"/>
     </row>
     <row r="26" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1">
-      <c r="A26" s="11"/>
-      <c r="B26" s="10"/>
-      <c r="C26" s="17"/>
-      <c r="D26" s="17"/>
-      <c r="E26" s="17"/>
-      <c r="F26" s="17"/>
-      <c r="G26" s="17"/>
-      <c r="H26" s="18"/>
+      <c r="A26" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="B26" s="20">
+        <v>45413</v>
+      </c>
+      <c r="C26" s="15"/>
+      <c r="D26" s="15"/>
+      <c r="E26" s="15"/>
+      <c r="F26" s="18"/>
+      <c r="G26" s="52"/>
+      <c r="H26" s="16"/>
       <c r="I26"/>
       <c r="J26"/>
       <c r="K26"/>
@@ -2122,17 +2261,19 @@
       <c r="AP26"/>
       <c r="AQ26"/>
     </row>
-    <row r="27" spans="1:43" s="2" customFormat="1" ht="17.399999999999999">
-      <c r="A27" s="32" t="s">
-        <v>20</v>
-      </c>
-      <c r="B27" s="33"/>
-      <c r="C27" s="33"/>
-      <c r="D27" s="33"/>
-      <c r="E27" s="33"/>
-      <c r="F27" s="33"/>
-      <c r="G27" s="33"/>
-      <c r="H27" s="34"/>
+    <row r="27" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1">
+      <c r="A27" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="B27" s="20">
+        <v>45413</v>
+      </c>
+      <c r="C27" s="15"/>
+      <c r="D27" s="18"/>
+      <c r="E27" s="15"/>
+      <c r="F27" s="15"/>
+      <c r="G27" s="15"/>
+      <c r="H27" s="16"/>
       <c r="I27"/>
       <c r="J27"/>
       <c r="K27"/>
@@ -2170,14 +2311,18 @@
       <c r="AQ27"/>
     </row>
     <row r="28" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1">
-      <c r="A28" s="11"/>
-      <c r="B28" s="10"/>
-      <c r="C28" s="17"/>
-      <c r="D28" s="17"/>
-      <c r="E28" s="17"/>
-      <c r="F28" s="17"/>
-      <c r="G28" s="17"/>
-      <c r="H28" s="18"/>
+      <c r="A28" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="B28" s="20">
+        <v>45413</v>
+      </c>
+      <c r="C28" s="15"/>
+      <c r="D28" s="15"/>
+      <c r="E28" s="15"/>
+      <c r="F28" s="15"/>
+      <c r="G28" s="18"/>
+      <c r="H28" s="16"/>
       <c r="I28"/>
       <c r="J28"/>
       <c r="K28"/>
@@ -2214,15 +2359,17 @@
       <c r="AP28"/>
       <c r="AQ28"/>
     </row>
-    <row r="29" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1">
-      <c r="A29" s="11"/>
-      <c r="B29" s="10"/>
-      <c r="C29" s="17"/>
-      <c r="D29" s="17"/>
-      <c r="E29" s="17"/>
-      <c r="F29" s="17"/>
-      <c r="G29" s="17"/>
-      <c r="H29" s="18"/>
+    <row r="29" spans="1:43" s="2" customFormat="1" ht="17.399999999999999">
+      <c r="A29" s="36" t="s">
+        <v>20</v>
+      </c>
+      <c r="B29" s="37"/>
+      <c r="C29" s="37"/>
+      <c r="D29" s="37"/>
+      <c r="E29" s="37"/>
+      <c r="F29" s="37"/>
+      <c r="G29" s="37"/>
+      <c r="H29" s="38"/>
       <c r="I29"/>
       <c r="J29"/>
       <c r="K29"/>
@@ -2260,14 +2407,18 @@
       <c r="AQ29"/>
     </row>
     <row r="30" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1">
-      <c r="A30" s="11"/>
-      <c r="B30" s="10"/>
-      <c r="C30" s="17"/>
-      <c r="D30" s="17"/>
-      <c r="E30" s="17"/>
-      <c r="F30" s="17"/>
-      <c r="G30" s="17"/>
-      <c r="H30" s="18"/>
+      <c r="A30" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="B30" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="C30" s="15"/>
+      <c r="D30" s="15"/>
+      <c r="E30" s="15"/>
+      <c r="F30" s="15"/>
+      <c r="G30" s="15"/>
+      <c r="H30" s="16"/>
       <c r="I30"/>
       <c r="J30"/>
       <c r="K30"/>
@@ -2305,14 +2456,18 @@
       <c r="AQ30"/>
     </row>
     <row r="31" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1">
-      <c r="A31" s="11"/>
-      <c r="B31" s="10"/>
-      <c r="C31" s="17"/>
-      <c r="D31" s="17"/>
-      <c r="E31" s="17"/>
-      <c r="F31" s="17"/>
-      <c r="G31" s="17"/>
-      <c r="H31" s="18"/>
+      <c r="A31" s="22" t="s">
+        <v>41</v>
+      </c>
+      <c r="B31" s="23" t="s">
+        <v>43</v>
+      </c>
+      <c r="C31" s="24"/>
+      <c r="D31" s="24"/>
+      <c r="E31" s="24"/>
+      <c r="F31" s="25"/>
+      <c r="G31" s="25"/>
+      <c r="H31" s="26"/>
       <c r="I31"/>
       <c r="J31"/>
       <c r="K31"/>
@@ -2350,14 +2505,18 @@
       <c r="AQ31"/>
     </row>
     <row r="32" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1">
-      <c r="A32" s="11"/>
-      <c r="B32" s="10"/>
-      <c r="C32" s="17"/>
-      <c r="D32" s="17"/>
-      <c r="E32" s="17"/>
-      <c r="F32" s="17"/>
-      <c r="G32" s="17"/>
-      <c r="H32" s="18"/>
+      <c r="A32" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="B32" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="C32" s="15"/>
+      <c r="D32" s="15"/>
+      <c r="E32" s="15"/>
+      <c r="F32" s="18"/>
+      <c r="G32" s="15"/>
+      <c r="H32" s="16"/>
       <c r="I32"/>
       <c r="J32"/>
       <c r="K32"/>
@@ -2395,14 +2554,18 @@
       <c r="AQ32"/>
     </row>
     <row r="33" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1">
-      <c r="A33" s="11"/>
-      <c r="B33" s="10"/>
-      <c r="C33" s="17"/>
-      <c r="D33" s="17"/>
-      <c r="E33" s="17"/>
-      <c r="F33" s="17"/>
-      <c r="G33" s="17"/>
-      <c r="H33" s="18"/>
+      <c r="A33" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="B33" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="C33" s="15"/>
+      <c r="D33" s="15"/>
+      <c r="E33" s="15"/>
+      <c r="F33" s="15"/>
+      <c r="G33" s="18"/>
+      <c r="H33" s="53"/>
       <c r="I33"/>
       <c r="J33"/>
       <c r="K33"/>
@@ -2439,15 +2602,19 @@
       <c r="AP33"/>
       <c r="AQ33"/>
     </row>
-    <row r="34" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" thickBot="1">
-      <c r="A34" s="12"/>
-      <c r="B34" s="13"/>
-      <c r="C34" s="19"/>
-      <c r="D34" s="19"/>
-      <c r="E34" s="19"/>
-      <c r="F34" s="19"/>
-      <c r="G34" s="19"/>
-      <c r="H34" s="20"/>
+    <row r="34" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1">
+      <c r="A34" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="B34" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="C34" s="18"/>
+      <c r="D34" s="18"/>
+      <c r="E34" s="15"/>
+      <c r="F34" s="18"/>
+      <c r="G34" s="15"/>
+      <c r="H34" s="16"/>
       <c r="I34"/>
       <c r="J34"/>
       <c r="K34"/>
@@ -2484,15 +2651,19 @@
       <c r="AP34"/>
       <c r="AQ34"/>
     </row>
-    <row r="35" spans="1:43" s="2" customFormat="1" ht="13.8">
-      <c r="A35" s="5"/>
-      <c r="B35" s="3"/>
-      <c r="C35" s="4"/>
-      <c r="D35" s="4"/>
-      <c r="E35" s="4"/>
-      <c r="F35" s="4"/>
-      <c r="G35" s="4"/>
-      <c r="H35" s="4"/>
+    <row r="35" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1">
+      <c r="A35" s="11" t="s">
+        <v>53</v>
+      </c>
+      <c r="B35" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="C35" s="15"/>
+      <c r="D35" s="15"/>
+      <c r="E35" s="15"/>
+      <c r="F35" s="15"/>
+      <c r="G35" s="18"/>
+      <c r="H35" s="16"/>
       <c r="I35"/>
       <c r="J35"/>
       <c r="K35"/>
@@ -2529,7 +2700,51 @@
       <c r="AP35"/>
       <c r="AQ35"/>
     </row>
-    <row r="36" spans="1:43" customFormat="1"/>
+    <row r="36" spans="1:43" s="2" customFormat="1" ht="13.8">
+      <c r="A36" s="5"/>
+      <c r="B36" s="3"/>
+      <c r="C36" s="4"/>
+      <c r="D36" s="4"/>
+      <c r="E36" s="4"/>
+      <c r="F36" s="4"/>
+      <c r="G36" s="4"/>
+      <c r="H36" s="4"/>
+      <c r="I36"/>
+      <c r="J36"/>
+      <c r="K36"/>
+      <c r="L36"/>
+      <c r="M36"/>
+      <c r="N36"/>
+      <c r="O36"/>
+      <c r="P36"/>
+      <c r="Q36"/>
+      <c r="R36"/>
+      <c r="S36"/>
+      <c r="T36"/>
+      <c r="U36"/>
+      <c r="V36"/>
+      <c r="W36"/>
+      <c r="X36"/>
+      <c r="Y36"/>
+      <c r="Z36"/>
+      <c r="AA36"/>
+      <c r="AB36"/>
+      <c r="AC36"/>
+      <c r="AD36"/>
+      <c r="AE36"/>
+      <c r="AF36"/>
+      <c r="AG36"/>
+      <c r="AH36"/>
+      <c r="AI36"/>
+      <c r="AJ36"/>
+      <c r="AK36"/>
+      <c r="AL36"/>
+      <c r="AM36"/>
+      <c r="AN36"/>
+      <c r="AO36"/>
+      <c r="AP36"/>
+      <c r="AQ36"/>
+    </row>
     <row r="37" spans="1:43" customFormat="1"/>
     <row r="38" spans="1:43" customFormat="1"/>
     <row r="39" spans="1:43" customFormat="1"/>
@@ -2575,6 +2790,7 @@
     <row r="79" customFormat="1"/>
     <row r="80" customFormat="1"/>
     <row r="81" customFormat="1"/>
+    <row r="82" customFormat="1"/>
   </sheetData>
   <mergeCells count="13">
     <mergeCell ref="G1:H1"/>
@@ -2585,8 +2801,8 @@
     <mergeCell ref="A6:A7"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A8:H8"/>
-    <mergeCell ref="A19:H19"/>
-    <mergeCell ref="A27:H27"/>
+    <mergeCell ref="A23:H23"/>
+    <mergeCell ref="A29:H29"/>
     <mergeCell ref="B6:B7"/>
     <mergeCell ref="A5:E5"/>
     <mergeCell ref="F5:H5"/>
@@ -2595,7 +2811,7 @@
   <hyperlinks>
     <hyperlink ref="A5:H5" r:id="rId1" display="Adresse URL du portfolio : htpps://juliengournay.fr" xr:uid="{95DEFDBE-0990-449B-BA48-5CE145C22ABA}"/>
   </hyperlinks>
-  <printOptions horizontalCentered="1" verticalCentered="1"/>
+  <printOptions horizontalCentered="1" verticalCentered="1" gridLines="1"/>
   <pageMargins left="0.19685039370078741" right="0.19685039370078741" top="0.19685039370078741" bottom="0.19685039370078741" header="0.51181102362204722" footer="0.51181102362204722"/>
   <pageSetup paperSize="9" scale="51" orientation="portrait" r:id="rId2"/>
   <headerFooter alignWithMargins="0"/>

</xml_diff>